<commit_message>
update 6 booking templates to latest user source (2026-08-14 空模板)
</commit_message>
<xml_diff>
--- a/templates/tpl_booking_mssnhsj6ni6f.xlsx
+++ b/templates/tpl_booking_mssnhsj6ni6f.xlsx
@@ -415,264 +415,6 @@
   </sheetPr>
   <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="164.5714285714286" customWidth="1" min="1" max="1"/>
-    <col width="231.5714285714286" customWidth="1" min="2" max="2"/>
-    <col width="505.8571428571428" customWidth="1" min="3" max="3"/>
-    <col width="597.2857142857143" customWidth="1" min="4" max="4"/>
-    <col width="576" customWidth="1" min="5" max="5"/>
-    <col width="538.1428571428571" customWidth="1" min="6" max="6"/>
-    <col width="67" customWidth="1" min="7" max="7"/>
-    <col width="585.1428571428571" customWidth="1" min="8" max="8"/>
-    <col width="579" customWidth="1" min="9" max="9"/>
-    <col width="329.1428571428572" customWidth="1" min="10" max="10"/>
-    <col width="329.1428571428572" customWidth="1" min="11" max="11"/>
-    <col width="329.1428571428572" customWidth="1" min="12" max="12"/>
-    <col width="329.1428571428572" customWidth="1" min="13" max="13"/>
-    <col width="329.1428571428572" customWidth="1" min="14" max="14"/>
-    <col width="329.1428571428572" customWidth="1" min="15" max="15"/>
-    <col width="329.1428571428572" customWidth="1" min="16" max="16"/>
-    <col width="329.1428571428572" customWidth="1" min="17" max="17"/>
-    <col width="329.1428571428572" customWidth="1" min="18" max="18"/>
-    <col width="329.1428571428572" customWidth="1" min="19" max="19"/>
-    <col width="329.1428571428572" customWidth="1" min="20" max="20"/>
-    <col width="329.1428571428572" customWidth="1" min="21" max="21"/>
-    <col width="329.1428571428572" customWidth="1" min="22" max="22"/>
-    <col width="329.1428571428572" customWidth="1" min="23" max="23"/>
-    <col width="329.1428571428572" customWidth="1" min="24" max="24"/>
-    <col width="329.1428571428572" customWidth="1" min="25" max="25"/>
-    <col width="329.1428571428572" customWidth="1" min="26" max="26"/>
-    <col width="329.1428571428572" customWidth="1" min="27" max="27"/>
-    <col width="329.1428571428572" customWidth="1" min="28" max="28"/>
-    <col width="329.1428571428572" customWidth="1" min="29" max="29"/>
-    <col width="329.1428571428572" customWidth="1" min="30" max="30"/>
-    <col width="329.1428571428572" customWidth="1" min="31" max="31"/>
-    <col width="329.1428571428572" customWidth="1" min="32" max="32"/>
-    <col width="329.1428571428572" customWidth="1" min="33" max="33"/>
-    <col width="329.1428571428572" customWidth="1" min="34" max="34"/>
-    <col width="329.1428571428572" customWidth="1" min="35" max="35"/>
-    <col width="329.1428571428572" customWidth="1" min="36" max="36"/>
-    <col width="329.1428571428572" customWidth="1" min="37" max="37"/>
-    <col width="329.1428571428572" customWidth="1" min="38" max="38"/>
-    <col width="329.1428571428572" customWidth="1" min="39" max="39"/>
-    <col width="329.1428571428572" customWidth="1" min="40" max="40"/>
-    <col width="329.1428571428572" customWidth="1" min="41" max="41"/>
-    <col width="329.1428571428572" customWidth="1" min="42" max="42"/>
-    <col width="329.1428571428572" customWidth="1" min="43" max="43"/>
-    <col width="329.1428571428572" customWidth="1" min="44" max="44"/>
-    <col width="329.1428571428572" customWidth="1" min="45" max="45"/>
-    <col width="329.1428571428572" customWidth="1" min="46" max="46"/>
-    <col width="329.1428571428572" customWidth="1" min="47" max="47"/>
-    <col width="329.1428571428572" customWidth="1" min="48" max="48"/>
-    <col width="329.1428571428572" customWidth="1" min="49" max="49"/>
-    <col width="329.1428571428572" customWidth="1" min="50" max="50"/>
-    <col width="329.1428571428572" customWidth="1" min="51" max="51"/>
-    <col width="329.1428571428572" customWidth="1" min="52" max="52"/>
-    <col width="329.1428571428572" customWidth="1" min="53" max="53"/>
-    <col width="329.1428571428572" customWidth="1" min="54" max="54"/>
-    <col width="329.1428571428572" customWidth="1" min="55" max="55"/>
-    <col width="329.1428571428572" customWidth="1" min="56" max="56"/>
-    <col width="329.1428571428572" customWidth="1" min="57" max="57"/>
-    <col width="329.1428571428572" customWidth="1" min="58" max="58"/>
-    <col width="329.1428571428572" customWidth="1" min="59" max="59"/>
-    <col width="329.1428571428572" customWidth="1" min="60" max="60"/>
-    <col width="329.1428571428572" customWidth="1" min="61" max="61"/>
-    <col width="329.1428571428572" customWidth="1" min="62" max="62"/>
-    <col width="329.1428571428572" customWidth="1" min="63" max="63"/>
-    <col width="329.1428571428572" customWidth="1" min="64" max="64"/>
-    <col width="329.1428571428572" customWidth="1" min="65" max="65"/>
-    <col width="329.1428571428572" customWidth="1" min="66" max="66"/>
-    <col width="329.1428571428572" customWidth="1" min="67" max="67"/>
-    <col width="329.1428571428572" customWidth="1" min="68" max="68"/>
-    <col width="329.1428571428572" customWidth="1" min="69" max="69"/>
-    <col width="329.1428571428572" customWidth="1" min="70" max="70"/>
-    <col width="329.1428571428572" customWidth="1" min="71" max="71"/>
-    <col width="329.1428571428572" customWidth="1" min="72" max="72"/>
-    <col width="329.1428571428572" customWidth="1" min="73" max="73"/>
-    <col width="329.1428571428572" customWidth="1" min="74" max="74"/>
-    <col width="329.1428571428572" customWidth="1" min="75" max="75"/>
-    <col width="329.1428571428572" customWidth="1" min="76" max="76"/>
-    <col width="329.1428571428572" customWidth="1" min="77" max="77"/>
-    <col width="329.1428571428572" customWidth="1" min="78" max="78"/>
-    <col width="329.1428571428572" customWidth="1" min="79" max="79"/>
-    <col width="329.1428571428572" customWidth="1" min="80" max="80"/>
-    <col width="329.1428571428572" customWidth="1" min="81" max="81"/>
-    <col width="329.1428571428572" customWidth="1" min="82" max="82"/>
-    <col width="329.1428571428572" customWidth="1" min="83" max="83"/>
-    <col width="329.1428571428572" customWidth="1" min="84" max="84"/>
-    <col width="329.1428571428572" customWidth="1" min="85" max="85"/>
-    <col width="329.1428571428572" customWidth="1" min="86" max="86"/>
-    <col width="329.1428571428572" customWidth="1" min="87" max="87"/>
-    <col width="329.1428571428572" customWidth="1" min="88" max="88"/>
-    <col width="329.1428571428572" customWidth="1" min="89" max="89"/>
-    <col width="329.1428571428572" customWidth="1" min="90" max="90"/>
-    <col width="329.1428571428572" customWidth="1" min="91" max="91"/>
-    <col width="329.1428571428572" customWidth="1" min="92" max="92"/>
-    <col width="329.1428571428572" customWidth="1" min="93" max="93"/>
-    <col width="329.1428571428572" customWidth="1" min="94" max="94"/>
-    <col width="329.1428571428572" customWidth="1" min="95" max="95"/>
-    <col width="329.1428571428572" customWidth="1" min="96" max="96"/>
-    <col width="329.1428571428572" customWidth="1" min="97" max="97"/>
-    <col width="329.1428571428572" customWidth="1" min="98" max="98"/>
-    <col width="329.1428571428572" customWidth="1" min="99" max="99"/>
-    <col width="329.1428571428572" customWidth="1" min="100" max="100"/>
-    <col width="329.1428571428572" customWidth="1" min="101" max="101"/>
-    <col width="329.1428571428572" customWidth="1" min="102" max="102"/>
-    <col width="329.1428571428572" customWidth="1" min="103" max="103"/>
-    <col width="329.1428571428572" customWidth="1" min="104" max="104"/>
-    <col width="329.1428571428572" customWidth="1" min="105" max="105"/>
-    <col width="329.1428571428572" customWidth="1" min="106" max="106"/>
-    <col width="329.1428571428572" customWidth="1" min="107" max="107"/>
-    <col width="329.1428571428572" customWidth="1" min="108" max="108"/>
-    <col width="329.1428571428572" customWidth="1" min="109" max="109"/>
-    <col width="329.1428571428572" customWidth="1" min="110" max="110"/>
-    <col width="329.1428571428572" customWidth="1" min="111" max="111"/>
-    <col width="329.1428571428572" customWidth="1" min="112" max="112"/>
-    <col width="329.1428571428572" customWidth="1" min="113" max="113"/>
-    <col width="329.1428571428572" customWidth="1" min="114" max="114"/>
-    <col width="329.1428571428572" customWidth="1" min="115" max="115"/>
-    <col width="329.1428571428572" customWidth="1" min="116" max="116"/>
-    <col width="329.1428571428572" customWidth="1" min="117" max="117"/>
-    <col width="329.1428571428572" customWidth="1" min="118" max="118"/>
-    <col width="329.1428571428572" customWidth="1" min="119" max="119"/>
-    <col width="329.1428571428572" customWidth="1" min="120" max="120"/>
-    <col width="329.1428571428572" customWidth="1" min="121" max="121"/>
-    <col width="329.1428571428572" customWidth="1" min="122" max="122"/>
-    <col width="329.1428571428572" customWidth="1" min="123" max="123"/>
-    <col width="329.1428571428572" customWidth="1" min="124" max="124"/>
-    <col width="329.1428571428572" customWidth="1" min="125" max="125"/>
-    <col width="329.1428571428572" customWidth="1" min="126" max="126"/>
-    <col width="329.1428571428572" customWidth="1" min="127" max="127"/>
-    <col width="329.1428571428572" customWidth="1" min="128" max="128"/>
-    <col width="329.1428571428572" customWidth="1" min="129" max="129"/>
-    <col width="329.1428571428572" customWidth="1" min="130" max="130"/>
-    <col width="329.1428571428572" customWidth="1" min="131" max="131"/>
-    <col width="329.1428571428572" customWidth="1" min="132" max="132"/>
-    <col width="329.1428571428572" customWidth="1" min="133" max="133"/>
-    <col width="329.1428571428572" customWidth="1" min="134" max="134"/>
-    <col width="329.1428571428572" customWidth="1" min="135" max="135"/>
-    <col width="329.1428571428572" customWidth="1" min="136" max="136"/>
-    <col width="329.1428571428572" customWidth="1" min="137" max="137"/>
-    <col width="329.1428571428572" customWidth="1" min="138" max="138"/>
-    <col width="329.1428571428572" customWidth="1" min="139" max="139"/>
-    <col width="329.1428571428572" customWidth="1" min="140" max="140"/>
-    <col width="329.1428571428572" customWidth="1" min="141" max="141"/>
-    <col width="329.1428571428572" customWidth="1" min="142" max="142"/>
-    <col width="329.1428571428572" customWidth="1" min="143" max="143"/>
-    <col width="329.1428571428572" customWidth="1" min="144" max="144"/>
-    <col width="329.1428571428572" customWidth="1" min="145" max="145"/>
-    <col width="329.1428571428572" customWidth="1" min="146" max="146"/>
-    <col width="329.1428571428572" customWidth="1" min="147" max="147"/>
-    <col width="329.1428571428572" customWidth="1" min="148" max="148"/>
-    <col width="329.1428571428572" customWidth="1" min="149" max="149"/>
-    <col width="329.1428571428572" customWidth="1" min="150" max="150"/>
-    <col width="329.1428571428572" customWidth="1" min="151" max="151"/>
-    <col width="329.1428571428572" customWidth="1" min="152" max="152"/>
-    <col width="329.1428571428572" customWidth="1" min="153" max="153"/>
-    <col width="329.1428571428572" customWidth="1" min="154" max="154"/>
-    <col width="329.1428571428572" customWidth="1" min="155" max="155"/>
-    <col width="329.1428571428572" customWidth="1" min="156" max="156"/>
-    <col width="329.1428571428572" customWidth="1" min="157" max="157"/>
-    <col width="329.1428571428572" customWidth="1" min="158" max="158"/>
-    <col width="329.1428571428572" customWidth="1" min="159" max="159"/>
-    <col width="329.1428571428572" customWidth="1" min="160" max="160"/>
-    <col width="329.1428571428572" customWidth="1" min="161" max="161"/>
-    <col width="329.1428571428572" customWidth="1" min="162" max="162"/>
-    <col width="329.1428571428572" customWidth="1" min="163" max="163"/>
-    <col width="329.1428571428572" customWidth="1" min="164" max="164"/>
-    <col width="329.1428571428572" customWidth="1" min="165" max="165"/>
-    <col width="329.1428571428572" customWidth="1" min="166" max="166"/>
-    <col width="329.1428571428572" customWidth="1" min="167" max="167"/>
-    <col width="329.1428571428572" customWidth="1" min="168" max="168"/>
-    <col width="329.1428571428572" customWidth="1" min="169" max="169"/>
-    <col width="329.1428571428572" customWidth="1" min="170" max="170"/>
-    <col width="329.1428571428572" customWidth="1" min="171" max="171"/>
-    <col width="329.1428571428572" customWidth="1" min="172" max="172"/>
-    <col width="329.1428571428572" customWidth="1" min="173" max="173"/>
-    <col width="329.1428571428572" customWidth="1" min="174" max="174"/>
-    <col width="329.1428571428572" customWidth="1" min="175" max="175"/>
-    <col width="329.1428571428572" customWidth="1" min="176" max="176"/>
-    <col width="329.1428571428572" customWidth="1" min="177" max="177"/>
-    <col width="329.1428571428572" customWidth="1" min="178" max="178"/>
-    <col width="329.1428571428572" customWidth="1" min="179" max="179"/>
-    <col width="329.1428571428572" customWidth="1" min="180" max="180"/>
-    <col width="329.1428571428572" customWidth="1" min="181" max="181"/>
-    <col width="329.1428571428572" customWidth="1" min="182" max="182"/>
-    <col width="329.1428571428572" customWidth="1" min="183" max="183"/>
-    <col width="329.1428571428572" customWidth="1" min="184" max="184"/>
-    <col width="329.1428571428572" customWidth="1" min="185" max="185"/>
-    <col width="329.1428571428572" customWidth="1" min="186" max="186"/>
-    <col width="329.1428571428572" customWidth="1" min="187" max="187"/>
-    <col width="329.1428571428572" customWidth="1" min="188" max="188"/>
-    <col width="329.1428571428572" customWidth="1" min="189" max="189"/>
-    <col width="329.1428571428572" customWidth="1" min="190" max="190"/>
-    <col width="329.1428571428572" customWidth="1" min="191" max="191"/>
-    <col width="329.1428571428572" customWidth="1" min="192" max="192"/>
-    <col width="329.1428571428572" customWidth="1" min="193" max="193"/>
-    <col width="329.1428571428572" customWidth="1" min="194" max="194"/>
-    <col width="329.1428571428572" customWidth="1" min="195" max="195"/>
-    <col width="329.1428571428572" customWidth="1" min="196" max="196"/>
-    <col width="329.1428571428572" customWidth="1" min="197" max="197"/>
-    <col width="329.1428571428572" customWidth="1" min="198" max="198"/>
-    <col width="329.1428571428572" customWidth="1" min="199" max="199"/>
-    <col width="329.1428571428572" customWidth="1" min="200" max="200"/>
-    <col width="329.1428571428572" customWidth="1" min="201" max="201"/>
-    <col width="329.1428571428572" customWidth="1" min="202" max="202"/>
-    <col width="329.1428571428572" customWidth="1" min="203" max="203"/>
-    <col width="329.1428571428572" customWidth="1" min="204" max="204"/>
-    <col width="329.1428571428572" customWidth="1" min="205" max="205"/>
-    <col width="329.1428571428572" customWidth="1" min="206" max="206"/>
-    <col width="329.1428571428572" customWidth="1" min="207" max="207"/>
-    <col width="329.1428571428572" customWidth="1" min="208" max="208"/>
-    <col width="329.1428571428572" customWidth="1" min="209" max="209"/>
-    <col width="329.1428571428572" customWidth="1" min="210" max="210"/>
-    <col width="329.1428571428572" customWidth="1" min="211" max="211"/>
-    <col width="329.1428571428572" customWidth="1" min="212" max="212"/>
-    <col width="329.1428571428572" customWidth="1" min="213" max="213"/>
-    <col width="329.1428571428572" customWidth="1" min="214" max="214"/>
-    <col width="329.1428571428572" customWidth="1" min="215" max="215"/>
-    <col width="329.1428571428572" customWidth="1" min="216" max="216"/>
-    <col width="329.1428571428572" customWidth="1" min="217" max="217"/>
-    <col width="329.1428571428572" customWidth="1" min="218" max="218"/>
-    <col width="329.1428571428572" customWidth="1" min="219" max="219"/>
-    <col width="329.1428571428572" customWidth="1" min="220" max="220"/>
-    <col width="329.1428571428572" customWidth="1" min="221" max="221"/>
-    <col width="329.1428571428572" customWidth="1" min="222" max="222"/>
-    <col width="329.1428571428572" customWidth="1" min="223" max="223"/>
-    <col width="329.1428571428572" customWidth="1" min="224" max="224"/>
-    <col width="329.1428571428572" customWidth="1" min="225" max="225"/>
-    <col width="329.1428571428572" customWidth="1" min="226" max="226"/>
-    <col width="329.1428571428572" customWidth="1" min="227" max="227"/>
-    <col width="329.1428571428572" customWidth="1" min="228" max="228"/>
-    <col width="329.1428571428572" customWidth="1" min="229" max="229"/>
-    <col width="329.1428571428572" customWidth="1" min="230" max="230"/>
-    <col width="329.1428571428572" customWidth="1" min="231" max="231"/>
-    <col width="329.1428571428572" customWidth="1" min="232" max="232"/>
-    <col width="329.1428571428572" customWidth="1" min="233" max="233"/>
-    <col width="329.1428571428572" customWidth="1" min="234" max="234"/>
-    <col width="329.1428571428572" customWidth="1" min="235" max="235"/>
-    <col width="329.1428571428572" customWidth="1" min="236" max="236"/>
-    <col width="329.1428571428572" customWidth="1" min="237" max="237"/>
-    <col width="329.1428571428572" customWidth="1" min="238" max="238"/>
-    <col width="329.1428571428572" customWidth="1" min="239" max="239"/>
-    <col width="329.1428571428572" customWidth="1" min="240" max="240"/>
-    <col width="329.1428571428572" customWidth="1" min="241" max="241"/>
-    <col width="329.1428571428572" customWidth="1" min="242" max="242"/>
-    <col width="329.1428571428572" customWidth="1" min="243" max="243"/>
-    <col width="329.1428571428572" customWidth="1" min="244" max="244"/>
-    <col width="329.1428571428572" customWidth="1" min="245" max="245"/>
-    <col width="329.1428571428572" customWidth="1" min="246" max="246"/>
-    <col width="329.1428571428572" customWidth="1" min="247" max="247"/>
-    <col width="329.1428571428572" customWidth="1" min="248" max="248"/>
-    <col width="329.1428571428572" customWidth="1" min="249" max="249"/>
-    <col width="329.1428571428572" customWidth="1" min="250" max="250"/>
-    <col width="329.1428571428572" customWidth="1" min="251" max="251"/>
-    <col width="329.1428571428572" customWidth="1" min="252" max="252"/>
-    <col width="329.1428571428572" customWidth="1" min="253" max="253"/>
-    <col width="329.1428571428572" customWidth="1" min="254" max="254"/>
-    <col width="329.1428571428572" customWidth="1" min="255" max="255"/>
-    <col width="329.1428571428572" customWidth="1" min="256" max="256"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -680,66 +422,179 @@
           <t>FROM:                                                         TO:</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+      <c r="F1" t="inlineStr"/>
+      <c r="G1" t="inlineStr"/>
+      <c r="H1" t="inlineStr"/>
+      <c r="I1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>*Shipper (托运人）:</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-    </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>*Consignee（收货人）</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t xml:space="preserve">深圳安海华南物流有限公司
 </t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>SHENZHEN ANHAI LOGISTICS CO.,LTD.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Attn:April</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>overseas01.sz@tjanhai.com</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t xml:space="preserve">Mob./Wechat:+86 130 7733 7519 </t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -747,23 +602,72 @@
           <t xml:space="preserve">*Notify Party （通知人） : </t>
         </is>
       </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>发票抬头(中文全称):</t>
         </is>
       </c>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
     <row r="19">
+      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>*Vessel/Voyage Number（船名或者截关日期）</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t xml:space="preserve">*Port of Loading </t>
@@ -779,19 +683,32 @@
           <t>*Port of Discharge</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>（卸货港）</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
     <row r="21">
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t xml:space="preserve">*Place of Receipt </t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>（收货地）</t>
@@ -812,14 +729,28 @@
           <t>Booking Confirmation Number</t>
         </is>
       </c>
-    </row>
-    <row r="22"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
     <row r="23">
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Marks &amp; Numbers</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Quantity</t>
@@ -830,6 +761,8 @@
           <t xml:space="preserve">                      * Description of Goods</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t xml:space="preserve">* Gross Weight </t>
@@ -842,11 +775,13 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t xml:space="preserve"> (唛头)</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>（数量）</t>
@@ -857,6 +792,8 @@
           <t xml:space="preserve">                            （货物描述）</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>（毛重 KGS）</t>
@@ -874,19 +811,95 @@
           <t>N/M</t>
         </is>
       </c>
-    </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+    </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>*TOTAL :  (       ) X20'GP,    (   ) X40'GP,    (     ) X40'HQ,(     ) X45'HQ,</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -894,24 +907,48 @@
           <t xml:space="preserve">       (      )Ocean freight Prepaid</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t xml:space="preserve">          (       )Ocean freight collect</t>
         </is>
       </c>
-    </row>
-    <row r="34"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+    </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
           <t>运费预付</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t xml:space="preserve">         运费到付</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -919,6 +956,9 @@
           <t xml:space="preserve">Remarks:                                                                  1.请(用英文)填完整以上托运单并回传我司, 内容务必正确.                                                                2.我司的付款制度为付款交单, 故请提早安排付费事宜, 以免因付款原因影响放单.                                  3.请提供详细的发票抬头, 以便我司出具发票.         4.未尽事宜, 请在双方合作中协议解决. </t>
         </is>
       </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>订舱托书注意事项:                                                1) 产品内如有任何电池类附件也请及时告知。请提供相应文件,如果无任何告知，默认为不含油和电池
@@ -926,61 +966,130 @@
 3)对于任何化工品/危险品的瞒报造成的一切后果和责任，都由委托方承担。</t>
         </is>
       </c>
-    </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+    </row>
     <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>*托运人签章:</t>
         </is>
       </c>
-    </row>
-    <row r="44"/>
-    <row r="45"/>
+      <c r="I43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+    </row>
     <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>日期(DATE):</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="A9:E13"/>
-    <mergeCell ref="E26:G29"/>
-    <mergeCell ref="E30:I31"/>
-    <mergeCell ref="A33:E34"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="D25:D29"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F33:I34"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A1:I2"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="A4:E7"/>
-    <mergeCell ref="A25:C28"/>
-    <mergeCell ref="A15:E18"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="E36:G44"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A36:D46"/>
-    <mergeCell ref="I25:I29"/>
-    <mergeCell ref="E22:F22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>